<commit_message>
Add column don_gia to exxcel file and edit logic import file
</commit_message>
<xml_diff>
--- a/public/samples/plates/tamnhua.xlsx
+++ b/public/samples/plates/tamnhua.xlsx
@@ -1,31 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leanhtu/Desktop/merge/project_freelance/KHO/KHO TẤM/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47CC8380-127F-C343-8B6F-07234835E67E}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1460" windowWidth="27240" windowHeight="14940" xr2:uid="{7B331964-EB66-944E-9FF5-F46C2638CDF3}"/>
+    <workbookView windowWidth="28800" windowHeight="12040"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="179021"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="57">
   <si>
     <t>Tồn</t>
   </si>
@@ -75,6 +64,9 @@
   </si>
   <si>
     <t>SL- m2</t>
+  </si>
+  <si>
+    <t>Đơn giá</t>
   </si>
   <si>
     <t>PLS P6NC 005</t>
@@ -203,29 +195,370 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="d&quot;/&quot;m&quot;/&quot;yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="6">
+    <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="d&quot;/&quot;m&quot;/&quot;yyyy"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -233,28 +566,314 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="60% - Accent6" xfId="1" builtinId="52"/>
+    <cellStyle name="40% - Accent6" xfId="2" builtinId="51"/>
+    <cellStyle name="60% - Accent5" xfId="3" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="4" builtinId="49"/>
+    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
+    <cellStyle name="20% - Accent5" xfId="6" builtinId="46"/>
+    <cellStyle name="60% - Accent4" xfId="7" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="8" builtinId="45"/>
+    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
+    <cellStyle name="Accent4" xfId="10" builtinId="41"/>
+    <cellStyle name="Linked Cell" xfId="11" builtinId="24"/>
+    <cellStyle name="40% - Accent3" xfId="12" builtinId="39"/>
+    <cellStyle name="60% - Accent2" xfId="13" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="14" builtinId="37"/>
+    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
+    <cellStyle name="20% - Accent2" xfId="16" builtinId="34"/>
+    <cellStyle name="Accent2" xfId="17" builtinId="33"/>
+    <cellStyle name="40% - Accent1" xfId="18" builtinId="31"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
+    <cellStyle name="Accent1" xfId="20" builtinId="29"/>
+    <cellStyle name="Neutral" xfId="21" builtinId="28"/>
+    <cellStyle name="60% - Accent1" xfId="22" builtinId="32"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="20% - Accent4" xfId="24" builtinId="42"/>
+    <cellStyle name="Total" xfId="25" builtinId="25"/>
+    <cellStyle name="Output" xfId="26" builtinId="21"/>
+    <cellStyle name="Currency" xfId="27" builtinId="4"/>
+    <cellStyle name="20% - Accent3" xfId="28" builtinId="38"/>
+    <cellStyle name="Note" xfId="29" builtinId="10"/>
+    <cellStyle name="Input" xfId="30" builtinId="20"/>
+    <cellStyle name="Heading 4" xfId="31" builtinId="19"/>
+    <cellStyle name="Calculation" xfId="32" builtinId="22"/>
+    <cellStyle name="Good" xfId="33" builtinId="26"/>
+    <cellStyle name="Heading 3" xfId="34" builtinId="18"/>
+    <cellStyle name="CExplanatory Text" xfId="35" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="36" builtinId="16"/>
+    <cellStyle name="Comma [0]" xfId="37" builtinId="6"/>
+    <cellStyle name="20% - Accent6" xfId="38" builtinId="50"/>
+    <cellStyle name="Title" xfId="39" builtinId="15"/>
+    <cellStyle name="Currency [0]" xfId="40" builtinId="7"/>
+    <cellStyle name="Warning Text" xfId="41" builtinId="11"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9"/>
+    <cellStyle name="Heading 2" xfId="43" builtinId="17"/>
+    <cellStyle name="Comma" xfId="44" builtinId="3"/>
+    <cellStyle name="Check Cell" xfId="45" builtinId="23"/>
+    <cellStyle name="60% - Accent3" xfId="46" builtinId="40"/>
+    <cellStyle name="Percent" xfId="47" builtinId="5"/>
+    <cellStyle name="Hyperlink" xfId="48" builtinId="8"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -303,7 +922,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -336,26 +955,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -388,23 +990,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -546,29 +1131,24 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C10F9C7-9341-FD49-BA10-C9E028868F93}">
-  <dimension ref="A1:O70"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:P70"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.8"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="3:14">
       <c r="C1" s="1"/>
-      <c r="J1" s="2"/>
-      <c r="M1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="M1" s="4"/>
       <c r="N1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -596,7 +1176,7 @@
       <c r="I2" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="K2" t="s">
@@ -605,28 +1185,31 @@
       <c r="L2" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="4" t="s">
         <v>13</v>
       </c>
       <c r="N2" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1">
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3">
         <v>1000</v>
@@ -637,110 +1220,110 @@
       <c r="I3">
         <v>1</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="3">
         <v>1.575</v>
       </c>
       <c r="K3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M3" s="4"/>
       <c r="N3">
         <v>1</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="3">
         <v>1.575</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
       </c>
       <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="2">
+        <v>180</v>
+      </c>
+      <c r="F4" s="2">
+        <v>660</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0.1188</v>
+      </c>
+      <c r="K4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L4" t="s">
+        <v>20</v>
+      </c>
+      <c r="M4" s="4"/>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4" s="3">
+        <v>0.1188</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
         <v>17</v>
-      </c>
-      <c r="E4" s="4">
-        <v>180</v>
-      </c>
-      <c r="F4" s="4">
-        <v>660</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4" s="2">
-        <v>0.1188</v>
-      </c>
-      <c r="K4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L4" t="s">
-        <v>19</v>
-      </c>
-      <c r="M4" s="3"/>
-      <c r="N4">
-        <v>1</v>
-      </c>
-      <c r="O4" s="2">
-        <v>0.1188</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
       </c>
       <c r="C5" s="1">
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="4">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2">
         <v>232</v>
       </c>
       <c r="I5">
         <v>4</v>
       </c>
-      <c r="J5" s="2">
-        <v>0.16900736000000002</v>
+      <c r="J5" s="3">
+        <v>0.16900736</v>
       </c>
       <c r="K5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L5" t="s">
-        <v>19</v>
-      </c>
-      <c r="M5" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M5" s="4"/>
       <c r="N5">
         <v>4</v>
       </c>
-      <c r="O5" s="2">
-        <v>0.16900736000000002</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O5" s="3">
+        <v>0.16900736</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="1">
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>620</v>
@@ -751,74 +1334,74 @@
       <c r="I6">
         <v>1</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="3">
         <v>0.62</v>
       </c>
       <c r="K6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L6" t="s">
-        <v>19</v>
-      </c>
-      <c r="M6" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M6" s="4"/>
       <c r="N6">
         <v>0</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1">
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7">
         <v>620</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="2">
         <v>900</v>
       </c>
       <c r="I7">
         <v>1</v>
       </c>
-      <c r="J7" s="2">
-        <v>0.55800000000000005</v>
+      <c r="J7" s="3">
+        <v>0.558</v>
       </c>
       <c r="K7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L7" t="s">
-        <v>19</v>
-      </c>
-      <c r="M7" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M7" s="4"/>
       <c r="N7">
         <v>1</v>
       </c>
-      <c r="O7" s="2">
-        <v>0.55800000000000005</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O7" s="3">
+        <v>0.558</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="1">
         <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8">
         <v>600</v>
@@ -829,74 +1412,74 @@
       <c r="I8">
         <v>1</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="3">
         <v>0.72</v>
       </c>
       <c r="K8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L8" t="s">
-        <v>19</v>
-      </c>
-      <c r="M8" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M8" s="4"/>
       <c r="N8">
         <v>1</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="3">
         <v>0.72</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1">
         <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E9">
         <v>500</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <v>800</v>
       </c>
       <c r="I9">
         <v>1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="3">
         <v>0.4</v>
       </c>
       <c r="K9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L9" t="s">
-        <v>19</v>
-      </c>
-      <c r="M9" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M9" s="4"/>
       <c r="N9">
         <v>0</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" s="1">
         <v>100</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E10">
         <v>380</v>
@@ -907,35 +1490,35 @@
       <c r="I10">
         <v>1</v>
       </c>
-      <c r="J10" s="2">
-        <v>0.39900000000000002</v>
+      <c r="J10" s="3">
+        <v>0.399</v>
       </c>
       <c r="K10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L10" t="s">
-        <v>19</v>
-      </c>
-      <c r="M10" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M10" s="4"/>
       <c r="N10">
         <v>1</v>
       </c>
-      <c r="O10" s="2">
-        <v>0.39900000000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O10" s="3">
+        <v>0.399</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1">
         <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E11">
         <v>540</v>
@@ -946,74 +1529,74 @@
       <c r="I11">
         <v>1</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="3">
         <v>0.54</v>
       </c>
       <c r="K11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L11" t="s">
-        <v>19</v>
-      </c>
-      <c r="M11" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M11" s="4"/>
       <c r="N11">
         <v>1</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11" s="3">
         <v>0.54</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1">
         <v>40</v>
       </c>
       <c r="D12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12">
         <v>260</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="2">
         <v>300</v>
       </c>
       <c r="I12">
         <v>1</v>
       </c>
-      <c r="J12" s="2">
-        <v>7.8E-2</v>
+      <c r="J12" s="3">
+        <v>0.078</v>
       </c>
       <c r="K12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L12" t="s">
-        <v>19</v>
-      </c>
-      <c r="M12" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M12" s="4"/>
       <c r="N12">
         <v>1</v>
       </c>
-      <c r="O12" s="2">
-        <v>7.8E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O12" s="3">
+        <v>0.078</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" s="1">
         <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13">
         <v>70</v>
@@ -1024,35 +1607,35 @@
       <c r="I13">
         <v>1</v>
       </c>
-      <c r="J13" s="2">
-        <v>7.0000000000000007E-2</v>
+      <c r="J13" s="3">
+        <v>0.07</v>
       </c>
       <c r="K13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L13" t="s">
-        <v>19</v>
-      </c>
-      <c r="M13" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M13" s="4"/>
       <c r="N13">
         <v>1</v>
       </c>
-      <c r="O13" s="2">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O13" s="3">
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
         <v>25</v>
-      </c>
-      <c r="B14" t="s">
-        <v>24</v>
       </c>
       <c r="C14" s="1">
         <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E14">
         <v>390</v>
@@ -1063,35 +1646,35 @@
       <c r="I14">
         <v>1</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="3">
         <v>0.39</v>
       </c>
       <c r="K14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L14" t="s">
-        <v>19</v>
-      </c>
-      <c r="M14" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M14" s="4"/>
       <c r="N14">
         <v>1</v>
       </c>
-      <c r="O14" s="2">
+      <c r="O14" s="3">
         <v>0.39</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C15" s="1">
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E15">
         <v>900</v>
@@ -1102,35 +1685,35 @@
       <c r="I15">
         <v>1</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="3">
         <v>2.7</v>
       </c>
       <c r="K15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L15" t="s">
-        <v>19</v>
-      </c>
-      <c r="M15" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M15" s="4"/>
       <c r="N15">
         <v>1</v>
       </c>
-      <c r="O15" s="2">
+      <c r="O15" s="3">
         <v>2.7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1">
         <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E16">
         <v>1000</v>
@@ -1141,113 +1724,113 @@
       <c r="I16">
         <v>1</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="3">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L16" t="s">
-        <v>19</v>
-      </c>
-      <c r="M16" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M16" s="4"/>
       <c r="N16">
         <v>0</v>
       </c>
-      <c r="O16" s="2">
+      <c r="O16" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C17" s="1">
         <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E17">
         <v>1000</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="2">
         <v>115</v>
       </c>
       <c r="I17">
         <v>1</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="3">
         <v>0.115</v>
       </c>
       <c r="K17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L17" t="s">
-        <v>19</v>
-      </c>
-      <c r="M17" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M17" s="4"/>
       <c r="N17">
         <v>1</v>
       </c>
-      <c r="O17" s="2">
+      <c r="O17" s="3">
         <v>0.115</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" s="1">
         <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E18">
         <v>500</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="2">
         <v>800</v>
       </c>
       <c r="I18">
         <v>1</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="3">
         <v>0.4</v>
       </c>
       <c r="K18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L18" t="s">
-        <v>19</v>
-      </c>
-      <c r="M18" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M18" s="4"/>
       <c r="N18">
         <v>0</v>
       </c>
-      <c r="O18" s="2">
+      <c r="O18" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" t="s">
         <v>30</v>
-      </c>
-      <c r="B19" t="s">
-        <v>29</v>
       </c>
       <c r="C19" s="1">
         <v>15</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E19">
         <v>1000</v>
@@ -1258,74 +1841,74 @@
       <c r="I19">
         <v>4</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="3">
         <v>8</v>
       </c>
       <c r="K19" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L19" t="s">
-        <v>19</v>
-      </c>
-      <c r="M19" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M19" s="4"/>
       <c r="N19">
         <v>4</v>
       </c>
-      <c r="O19" s="2">
+      <c r="O19" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15">
       <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
         <v>30</v>
-      </c>
-      <c r="B20" t="s">
-        <v>29</v>
       </c>
       <c r="C20" s="1">
         <v>15</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E20">
         <v>1000</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="2">
         <v>800</v>
       </c>
       <c r="I20">
         <v>1</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="3">
         <v>0.8</v>
       </c>
       <c r="K20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L20" t="s">
-        <v>19</v>
-      </c>
-      <c r="M20" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M20" s="4"/>
       <c r="N20">
         <v>1</v>
       </c>
-      <c r="O20" s="2">
+      <c r="O20" s="3">
         <v>0.8</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15">
       <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" t="s">
         <v>30</v>
-      </c>
-      <c r="B21" t="s">
-        <v>29</v>
       </c>
       <c r="C21" s="1">
         <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E21">
         <v>60</v>
@@ -1336,35 +1919,35 @@
       <c r="I21">
         <v>4</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="3">
         <v>0.48</v>
       </c>
       <c r="K21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L21" t="s">
-        <v>19</v>
-      </c>
-      <c r="M21" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M21" s="4"/>
       <c r="N21">
         <v>4</v>
       </c>
-      <c r="O21" s="2">
+      <c r="O21" s="3">
         <v>0.48</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C22" s="1">
         <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E22">
         <v>1000</v>
@@ -1375,35 +1958,35 @@
       <c r="I22">
         <v>9</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="3">
         <v>18</v>
       </c>
       <c r="K22" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L22" t="s">
-        <v>19</v>
-      </c>
-      <c r="M22" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M22" s="4"/>
       <c r="N22">
         <v>0</v>
       </c>
-      <c r="O22" s="2">
+      <c r="O22" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C23" s="1">
         <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E23">
         <v>500</v>
@@ -1414,35 +1997,35 @@
       <c r="I23">
         <v>1</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="3">
         <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L23" t="s">
-        <v>19</v>
-      </c>
-      <c r="M23" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M23" s="4"/>
       <c r="N23">
         <v>0</v>
       </c>
-      <c r="O23" s="2">
+      <c r="O23" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C24" s="1">
         <v>20</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E24">
         <v>500</v>
@@ -1453,35 +2036,35 @@
       <c r="I24">
         <v>1</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="3">
         <v>0.75</v>
       </c>
       <c r="K24" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L24" t="s">
-        <v>19</v>
-      </c>
-      <c r="M24" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M24" s="4"/>
       <c r="N24">
         <v>1</v>
       </c>
-      <c r="O24" s="2">
+      <c r="O24" s="3">
         <v>0.75</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C25" s="1">
         <v>20</v>
       </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E25">
         <v>460</v>
@@ -1492,35 +2075,35 @@
       <c r="I25">
         <v>1</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="3">
         <v>0.92</v>
       </c>
       <c r="K25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L25" t="s">
-        <v>19</v>
-      </c>
-      <c r="M25" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M25" s="4"/>
       <c r="N25">
         <v>0</v>
       </c>
-      <c r="O25" s="2">
+      <c r="O25" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C26" s="1">
         <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E26">
         <v>340</v>
@@ -1531,35 +2114,35 @@
       <c r="I26">
         <v>1</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="3">
         <v>0.68</v>
       </c>
       <c r="K26" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L26" t="s">
-        <v>19</v>
-      </c>
-      <c r="M26" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M26" s="4"/>
       <c r="N26">
         <v>0</v>
       </c>
-      <c r="O26" s="2">
+      <c r="O26" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C27" s="1">
         <v>20</v>
       </c>
       <c r="D27" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E27">
         <v>200</v>
@@ -1570,35 +2153,35 @@
       <c r="I27">
         <v>1</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="3">
         <v>0.4</v>
       </c>
       <c r="K27" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L27" t="s">
-        <v>19</v>
-      </c>
-      <c r="M27" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M27" s="4"/>
       <c r="N27">
         <v>0</v>
       </c>
-      <c r="O27" s="2">
+      <c r="O27" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C28" s="1">
         <v>20</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E28">
         <v>60</v>
@@ -1609,35 +2192,35 @@
       <c r="I28">
         <v>18</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="3">
         <v>2.16</v>
       </c>
       <c r="K28" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L28" t="s">
-        <v>19</v>
-      </c>
-      <c r="M28" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M28" s="4"/>
       <c r="N28">
         <v>8</v>
       </c>
-      <c r="O28" s="2">
+      <c r="O28" s="3">
         <v>0.96</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C29" s="1">
         <v>20</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E29">
         <v>680</v>
@@ -1648,35 +2231,35 @@
       <c r="I29">
         <v>1</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="3">
         <v>2.04</v>
       </c>
       <c r="K29" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L29" t="s">
-        <v>19</v>
-      </c>
-      <c r="M29" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M29" s="4"/>
       <c r="N29">
         <v>1</v>
       </c>
-      <c r="O29" s="2">
+      <c r="O29" s="3">
         <v>2.04</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C30" s="1">
         <v>20</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E30">
         <v>1200</v>
@@ -1687,35 +2270,35 @@
       <c r="I30">
         <v>1</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="3">
         <v>1.248</v>
       </c>
       <c r="K30" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L30" t="s">
-        <v>19</v>
-      </c>
-      <c r="M30" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M30" s="4"/>
       <c r="N30">
         <v>1</v>
       </c>
-      <c r="O30" s="2">
+      <c r="O30" s="3">
         <v>1.248</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C31" s="1">
         <v>25</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E31">
         <v>1000</v>
@@ -1726,35 +2309,35 @@
       <c r="I31">
         <v>2</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="3">
         <v>4</v>
       </c>
       <c r="K31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L31" t="s">
-        <v>19</v>
-      </c>
-      <c r="M31" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M31" s="4"/>
       <c r="N31">
         <v>2</v>
       </c>
-      <c r="O31" s="2">
+      <c r="O31" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C32" s="1">
         <v>25</v>
       </c>
       <c r="D32" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E32">
         <v>1000</v>
@@ -1765,35 +2348,35 @@
       <c r="I32">
         <v>1</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="3">
         <v>2</v>
       </c>
       <c r="K32" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L32" t="s">
-        <v>19</v>
-      </c>
-      <c r="M32" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M32" s="4"/>
       <c r="N32">
         <v>1</v>
       </c>
-      <c r="O32" s="2">
+      <c r="O32" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C33" s="1">
         <v>50</v>
       </c>
       <c r="D33" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E33">
         <v>1000</v>
@@ -1804,35 +2387,35 @@
       <c r="I33">
         <v>1</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="3">
         <v>1.23</v>
       </c>
       <c r="K33" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L33" t="s">
-        <v>19</v>
-      </c>
-      <c r="M33" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M33" s="4"/>
       <c r="N33">
         <v>1</v>
       </c>
-      <c r="O33" s="2">
+      <c r="O33" s="3">
         <v>1.23</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C34" s="1">
         <v>50</v>
       </c>
       <c r="D34" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E34">
         <v>1230</v>
@@ -1843,230 +2426,230 @@
       <c r="I34">
         <v>1</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="3">
         <v>2.0787</v>
       </c>
       <c r="K34" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L34" t="s">
-        <v>19</v>
-      </c>
-      <c r="M34" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M34" s="4"/>
       <c r="N34">
         <v>1</v>
       </c>
-      <c r="O34" s="2">
+      <c r="O34" s="3">
         <v>2.0787</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C35" s="1">
         <v>50</v>
       </c>
       <c r="D35" t="s">
-        <v>17</v>
-      </c>
-      <c r="E35" s="4">
+        <v>18</v>
+      </c>
+      <c r="E35" s="2">
         <v>600</v>
       </c>
-      <c r="F35" s="4">
+      <c r="F35" s="2">
         <v>430</v>
       </c>
       <c r="I35">
         <v>1</v>
       </c>
-      <c r="J35" s="2">
-        <v>0.25800000000000001</v>
+      <c r="J35" s="3">
+        <v>0.258</v>
       </c>
       <c r="K35" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L35" t="s">
-        <v>19</v>
-      </c>
-      <c r="M35" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M35" s="4"/>
       <c r="N35">
         <v>1</v>
       </c>
-      <c r="O35" s="2">
-        <v>0.25800000000000001</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O35" s="3">
+        <v>0.258</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C36" s="1">
         <v>50</v>
       </c>
       <c r="D36" t="s">
-        <v>17</v>
-      </c>
-      <c r="E36" s="4">
+        <v>18</v>
+      </c>
+      <c r="E36" s="2">
         <v>300</v>
       </c>
-      <c r="F36" s="4">
+      <c r="F36" s="2">
         <v>200</v>
       </c>
       <c r="I36">
         <v>1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="3">
         <v>0.06</v>
       </c>
       <c r="K36" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L36" t="s">
-        <v>19</v>
-      </c>
-      <c r="M36" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M36" s="4"/>
       <c r="N36">
         <v>1</v>
       </c>
-      <c r="O36" s="2">
+      <c r="O36" s="3">
         <v>0.06</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C37" s="1">
         <v>50</v>
       </c>
       <c r="D37" t="s">
-        <v>17</v>
-      </c>
-      <c r="E37" s="4">
+        <v>18</v>
+      </c>
+      <c r="E37" s="2">
         <v>280</v>
       </c>
-      <c r="F37" s="4">
+      <c r="F37" s="2">
         <v>200</v>
       </c>
       <c r="I37">
         <v>1</v>
       </c>
-      <c r="J37" s="2">
-        <v>5.6000000000000001E-2</v>
+      <c r="J37" s="3">
+        <v>0.056</v>
       </c>
       <c r="K37" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L37" t="s">
-        <v>19</v>
-      </c>
-      <c r="M37" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M37" s="4"/>
       <c r="N37">
         <v>1</v>
       </c>
-      <c r="O37" s="2">
-        <v>5.6000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O37" s="3">
+        <v>0.056</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C38" s="1">
         <v>50</v>
       </c>
       <c r="D38" t="s">
-        <v>17</v>
-      </c>
-      <c r="E38" s="4">
+        <v>18</v>
+      </c>
+      <c r="E38" s="2">
         <v>180</v>
       </c>
-      <c r="F38" s="4">
+      <c r="F38" s="2">
         <v>300</v>
       </c>
       <c r="I38">
         <v>1</v>
       </c>
-      <c r="J38" s="2">
-        <v>5.3999999999999999E-2</v>
+      <c r="J38" s="3">
+        <v>0.054</v>
       </c>
       <c r="K38" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L38" t="s">
-        <v>19</v>
-      </c>
-      <c r="M38" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M38" s="4"/>
       <c r="N38">
         <v>1</v>
       </c>
-      <c r="O38" s="2">
-        <v>5.3999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O38" s="3">
+        <v>0.054</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15">
       <c r="A39" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B39" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C39" s="1">
         <v>50</v>
       </c>
       <c r="D39" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" s="4">
+        <v>18</v>
+      </c>
+      <c r="E39" s="2">
         <v>700</v>
       </c>
-      <c r="F39" s="4">
+      <c r="F39" s="2">
         <v>140</v>
       </c>
       <c r="I39">
         <v>1</v>
       </c>
-      <c r="J39" s="2">
-        <v>9.8000000000000004E-2</v>
+      <c r="J39" s="3">
+        <v>0.098</v>
       </c>
       <c r="K39" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L39" t="s">
-        <v>19</v>
-      </c>
-      <c r="M39" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M39" s="4"/>
       <c r="N39">
         <v>1</v>
       </c>
-      <c r="O39" s="2">
-        <v>9.8000000000000004E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O39" s="3">
+        <v>0.098</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C40" s="1">
         <v>80</v>
       </c>
       <c r="D40" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E40">
         <v>1000</v>
@@ -2077,35 +2660,35 @@
       <c r="I40">
         <v>1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="3">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L40" t="s">
-        <v>19</v>
-      </c>
-      <c r="M40" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M40" s="4"/>
       <c r="N40">
         <v>1</v>
       </c>
-      <c r="O40" s="2">
+      <c r="O40" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C41" s="1">
         <v>15</v>
       </c>
       <c r="D41" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E41">
         <v>1000</v>
@@ -2116,35 +2699,35 @@
       <c r="I41">
         <v>5</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="3">
         <v>10</v>
       </c>
       <c r="K41" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L41" t="s">
-        <v>19</v>
-      </c>
-      <c r="M41" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M41" s="4"/>
       <c r="N41">
         <v>5</v>
       </c>
-      <c r="O41" s="2">
+      <c r="O41" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C42" s="1">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E42">
         <v>1300</v>
@@ -2155,35 +2738,35 @@
       <c r="I42">
         <v>1</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="3">
         <v>65</v>
       </c>
       <c r="K42" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L42" t="s">
-        <v>19</v>
-      </c>
-      <c r="M42" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M42" s="4"/>
       <c r="N42">
         <v>1</v>
       </c>
-      <c r="O42" s="2">
+      <c r="O42" s="3">
         <v>65</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C43" s="1">
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E43">
         <v>1000</v>
@@ -2194,35 +2777,35 @@
       <c r="I43">
         <v>1</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="3">
         <v>2</v>
       </c>
       <c r="K43" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L43" t="s">
-        <v>19</v>
-      </c>
-      <c r="M43" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M43" s="4"/>
       <c r="N43">
         <v>1</v>
       </c>
-      <c r="O43" s="2">
+      <c r="O43" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C44" s="1">
         <v>5</v>
       </c>
       <c r="D44" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E44">
         <v>1000</v>
@@ -2233,35 +2816,35 @@
       <c r="I44">
         <v>1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="3">
         <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L44" t="s">
-        <v>19</v>
-      </c>
-      <c r="M44" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M44" s="4"/>
       <c r="N44">
         <v>1</v>
       </c>
-      <c r="O44" s="2">
+      <c r="O44" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C45" s="1">
         <v>10</v>
       </c>
       <c r="D45" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E45">
         <v>330</v>
@@ -2272,35 +2855,35 @@
       <c r="I45">
         <v>1</v>
       </c>
-      <c r="J45" s="2">
-        <v>0.12540000000000001</v>
+      <c r="J45" s="3">
+        <v>0.1254</v>
       </c>
       <c r="K45" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L45" t="s">
-        <v>19</v>
-      </c>
-      <c r="M45" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M45" s="4"/>
       <c r="N45">
         <v>1</v>
       </c>
-      <c r="O45" s="2">
-        <v>0.12540000000000001</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O45" s="3">
+        <v>0.1254</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C46" s="1">
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E46">
         <v>250</v>
@@ -2311,37 +2894,37 @@
       <c r="I46">
         <v>1</v>
       </c>
-      <c r="J46" s="2">
-        <v>5.9499999999999997E-2</v>
+      <c r="J46" s="3">
+        <v>0.0595</v>
       </c>
       <c r="K46" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L46" t="s">
-        <v>19</v>
-      </c>
-      <c r="M46" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M46" s="4"/>
       <c r="N46">
         <v>1</v>
       </c>
-      <c r="O46" s="2">
-        <v>5.9499999999999997E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O46" s="3">
+        <v>0.0595</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15">
       <c r="A47" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C47" s="1">
         <v>70</v>
       </c>
       <c r="D47" t="s">
-        <v>17</v>
-      </c>
-      <c r="E47" s="4">
+        <v>18</v>
+      </c>
+      <c r="E47" s="2">
         <v>600</v>
       </c>
       <c r="F47">
@@ -2350,113 +2933,113 @@
       <c r="I47">
         <v>7</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="3">
         <v>5.04</v>
       </c>
       <c r="K47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L47" t="s">
-        <v>19</v>
-      </c>
-      <c r="M47" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M47" s="4"/>
       <c r="N47">
         <v>0</v>
       </c>
-      <c r="O47" s="2">
+      <c r="O47" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B48" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C48" s="1">
         <v>70</v>
       </c>
       <c r="D48" t="s">
-        <v>17</v>
-      </c>
-      <c r="E48" s="4">
+        <v>18</v>
+      </c>
+      <c r="E48" s="2">
         <v>300</v>
       </c>
-      <c r="F48" s="4">
+      <c r="F48" s="2">
         <v>350</v>
       </c>
       <c r="I48">
         <v>1</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="3">
         <v>0.105</v>
       </c>
       <c r="K48" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L48" t="s">
-        <v>19</v>
-      </c>
-      <c r="M48" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M48" s="4"/>
       <c r="N48">
         <v>0</v>
       </c>
-      <c r="O48" s="2">
+      <c r="O48" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C49" s="1">
         <v>70</v>
       </c>
       <c r="D49" t="s">
-        <v>17</v>
-      </c>
-      <c r="E49" s="4">
+        <v>18</v>
+      </c>
+      <c r="E49" s="2">
         <v>200</v>
       </c>
-      <c r="F49" s="4">
+      <c r="F49" s="2">
         <v>480</v>
       </c>
       <c r="I49">
         <v>1</v>
       </c>
-      <c r="J49" s="2">
-        <v>9.6000000000000002E-2</v>
+      <c r="J49" s="3">
+        <v>0.096</v>
       </c>
       <c r="K49" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L49" t="s">
-        <v>19</v>
-      </c>
-      <c r="M49" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="M49" s="4"/>
       <c r="N49">
         <v>0</v>
       </c>
-      <c r="O49" s="2">
+      <c r="O49" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C50" s="1">
         <v>70</v>
       </c>
       <c r="D50" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E50">
         <v>1000</v>
@@ -2467,37 +3050,37 @@
       <c r="I50">
         <v>5</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="3">
         <v>10</v>
       </c>
       <c r="K50" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L50" t="s">
-        <v>19</v>
-      </c>
-      <c r="M50" s="3">
+        <v>20</v>
+      </c>
+      <c r="M50" s="4">
         <v>44391</v>
       </c>
       <c r="N50">
         <v>1</v>
       </c>
-      <c r="O50" s="2">
+      <c r="O50" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15">
       <c r="A51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B51" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C51" s="1">
         <v>12</v>
       </c>
       <c r="D51" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E51">
         <v>500</v>
@@ -2508,37 +3091,37 @@
       <c r="I51">
         <v>1</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="3">
         <v>1</v>
       </c>
       <c r="K51" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L51">
         <v>2101819</v>
       </c>
-      <c r="M51" s="3">
+      <c r="M51" s="4">
         <v>44459</v>
       </c>
       <c r="N51">
         <v>1</v>
       </c>
-      <c r="O51" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O51" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15">
       <c r="A52" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C52" s="1">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E52">
         <v>350</v>
@@ -2549,37 +3132,37 @@
       <c r="I52">
         <v>1</v>
       </c>
-      <c r="J52" s="2">
-        <v>0.17499999999999999</v>
+      <c r="J52" s="3">
+        <v>0.175</v>
       </c>
       <c r="K52" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L52">
         <v>2101819</v>
       </c>
-      <c r="M52" s="3">
+      <c r="M52" s="4">
         <v>44459</v>
       </c>
       <c r="N52">
         <v>0</v>
       </c>
-      <c r="O52" s="2">
+      <c r="O52" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15">
       <c r="A53" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B53" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C53" s="1">
         <v>12</v>
       </c>
       <c r="D53" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E53">
         <v>50</v>
@@ -2590,37 +3173,37 @@
       <c r="I53">
         <v>1</v>
       </c>
-      <c r="J53" s="2">
-        <v>1.2500000000000001E-2</v>
+      <c r="J53" s="3">
+        <v>0.0125</v>
       </c>
       <c r="K53" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L53">
         <v>2101819</v>
       </c>
-      <c r="M53" s="3">
+      <c r="M53" s="4">
         <v>44459</v>
       </c>
       <c r="N53">
         <v>1</v>
       </c>
-      <c r="O53" s="2">
-        <v>1.2500000000000001E-2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O53" s="3">
+        <v>0.0125</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15">
       <c r="A54" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B54" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C54" s="1">
         <v>70</v>
       </c>
       <c r="D54" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E54">
         <v>1000</v>
@@ -2631,37 +3214,37 @@
       <c r="I54">
         <v>1</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="3">
         <v>1.5</v>
       </c>
       <c r="K54" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L54">
         <v>2101038</v>
       </c>
-      <c r="M54" s="3">
+      <c r="M54" s="4">
         <v>44336</v>
       </c>
       <c r="N54">
         <v>0</v>
       </c>
-      <c r="O54" s="2">
+      <c r="O54" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:15">
       <c r="A55" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B55" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C55" s="1">
         <v>20</v>
       </c>
       <c r="D55" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E55">
         <v>40</v>
@@ -2672,37 +3255,37 @@
       <c r="I55">
         <v>1</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="3">
         <v>0.08</v>
       </c>
       <c r="K55" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L55">
         <v>2101888</v>
       </c>
-      <c r="M55" s="3">
+      <c r="M55" s="4">
         <v>44473</v>
       </c>
       <c r="N55">
         <v>1</v>
       </c>
-      <c r="O55" s="2">
+      <c r="O55" s="3">
         <v>0.08</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15">
       <c r="A56" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B56" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C56" s="1">
         <v>12</v>
       </c>
       <c r="D56" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E56">
         <v>350</v>
@@ -2713,37 +3296,37 @@
       <c r="I56">
         <v>1</v>
       </c>
-      <c r="J56" s="2">
-        <v>9.4500000000000001E-2</v>
+      <c r="J56" s="3">
+        <v>0.0945</v>
       </c>
       <c r="K56" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L56">
         <v>2102360</v>
       </c>
-      <c r="M56" s="3">
+      <c r="M56" s="4">
         <v>44531</v>
       </c>
       <c r="N56">
         <v>1</v>
       </c>
-      <c r="O56" s="2">
-        <v>9.4500000000000001E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O56" s="3">
+        <v>0.0945</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15">
       <c r="A57" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B57" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C57" s="1">
         <v>12</v>
       </c>
       <c r="D57" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E57">
         <v>105</v>
@@ -2751,37 +3334,37 @@
       <c r="I57">
         <v>2</v>
       </c>
-      <c r="J57" s="2">
-        <v>1.7309250000000002E-2</v>
+      <c r="J57" s="3">
+        <v>0.01730925</v>
       </c>
       <c r="K57" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L57">
         <v>2102360</v>
       </c>
-      <c r="M57" s="3">
+      <c r="M57" s="4">
         <v>44531</v>
       </c>
       <c r="N57">
         <v>2</v>
       </c>
-      <c r="O57" s="2">
-        <v>1.7309250000000002E-2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O57" s="3">
+        <v>0.01730925</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15">
       <c r="A58" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B58" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C58" s="1">
         <v>10</v>
       </c>
       <c r="D58" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E58">
         <v>620</v>
@@ -2792,37 +3375,37 @@
       <c r="I58">
         <v>1</v>
       </c>
-      <c r="J58" s="2">
-        <v>0.55800000000000005</v>
+      <c r="J58" s="3">
+        <v>0.558</v>
       </c>
       <c r="K58" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L58">
         <v>2102370</v>
       </c>
-      <c r="M58" s="3">
+      <c r="M58" s="4">
         <v>44532</v>
       </c>
       <c r="N58">
         <v>0</v>
       </c>
-      <c r="O58" s="2">
+      <c r="O58" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:15">
       <c r="A59" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B59" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C59" s="1">
         <v>10</v>
       </c>
       <c r="D59" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E59">
         <v>80</v>
@@ -2833,37 +3416,37 @@
       <c r="I59">
         <v>1</v>
       </c>
-      <c r="J59" s="2">
-        <v>2.1600000000000001E-2</v>
+      <c r="J59" s="3">
+        <v>0.0216</v>
       </c>
       <c r="K59" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L59">
         <v>2102370</v>
       </c>
-      <c r="M59" s="3">
+      <c r="M59" s="4">
         <v>44532</v>
       </c>
       <c r="N59">
         <v>0</v>
       </c>
-      <c r="O59" s="2">
+      <c r="O59" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:15">
       <c r="A60" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B60" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C60" s="1">
         <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E60">
         <v>620</v>
@@ -2874,37 +3457,37 @@
       <c r="I60">
         <v>1</v>
       </c>
-      <c r="J60" s="2">
-        <v>0.40920000000000001</v>
+      <c r="J60" s="3">
+        <v>0.4092</v>
       </c>
       <c r="K60" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L60">
         <v>2102558</v>
       </c>
-      <c r="M60" s="3">
+      <c r="M60" s="4">
         <v>44559</v>
       </c>
       <c r="N60">
         <v>1</v>
       </c>
-      <c r="O60" s="2">
-        <v>0.40920000000000001</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O60" s="3">
+        <v>0.4092</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15">
       <c r="A61" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B61" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C61" s="1">
         <v>10</v>
       </c>
       <c r="D61" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E61">
         <v>170</v>
@@ -2915,37 +3498,37 @@
       <c r="I61">
         <v>1</v>
       </c>
-      <c r="J61" s="2">
-        <v>4.5900000000000003E-2</v>
+      <c r="J61" s="3">
+        <v>0.0459</v>
       </c>
       <c r="K61" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L61">
         <v>2102558</v>
       </c>
-      <c r="M61" s="3">
+      <c r="M61" s="4">
         <v>44559</v>
       </c>
       <c r="N61">
         <v>0</v>
       </c>
-      <c r="O61" s="2">
+      <c r="O61" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:15">
       <c r="A62" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B62" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C62" s="1">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E62">
         <v>80</v>
@@ -2956,37 +3539,37 @@
       <c r="I62">
         <v>1</v>
       </c>
-      <c r="J62" s="2">
-        <v>8.0000000000000002E-3</v>
+      <c r="J62" s="3">
+        <v>0.008</v>
       </c>
       <c r="K62" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L62">
         <v>2102432</v>
       </c>
-      <c r="M62" s="3">
+      <c r="M62" s="4">
         <v>44540</v>
       </c>
       <c r="N62">
         <v>0</v>
       </c>
-      <c r="O62" s="2">
+      <c r="O62" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:15">
       <c r="A63" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B63" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C63" s="1">
         <v>20</v>
       </c>
       <c r="D63" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E63">
         <v>1490</v>
@@ -2997,37 +3580,37 @@
       <c r="I63">
         <v>42</v>
       </c>
-      <c r="J63" s="2">
-        <v>155.82420000000002</v>
+      <c r="J63" s="3">
+        <v>155.8242</v>
       </c>
       <c r="K63" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L63" t="s">
-        <v>19</v>
-      </c>
-      <c r="M63" s="3">
+        <v>20</v>
+      </c>
+      <c r="M63" s="4">
         <v>44657</v>
       </c>
       <c r="N63">
         <v>0</v>
       </c>
-      <c r="O63" s="2">
+      <c r="O63" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:15">
       <c r="A64" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B64" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C64" s="1">
         <v>20</v>
       </c>
       <c r="D64" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E64">
         <v>120</v>
@@ -3038,37 +3621,37 @@
       <c r="I64">
         <v>1</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="3">
         <v>0.24</v>
       </c>
       <c r="K64" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L64">
         <v>2201498</v>
       </c>
-      <c r="M64" s="3">
+      <c r="M64" s="4">
         <v>44733</v>
       </c>
       <c r="N64">
         <v>1</v>
       </c>
-      <c r="O64" s="2">
+      <c r="O64" s="3">
         <v>0.24</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:15">
       <c r="A65" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B65" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C65" s="1">
         <v>10</v>
       </c>
       <c r="D65" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E65">
         <v>500</v>
@@ -3079,37 +3662,37 @@
       <c r="I65">
         <v>1</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="3">
         <v>0.36</v>
       </c>
       <c r="K65" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L65">
         <v>2202458</v>
       </c>
-      <c r="M65" s="3">
+      <c r="M65" s="4">
         <v>44830</v>
       </c>
       <c r="N65">
         <v>1</v>
       </c>
-      <c r="O65" s="2">
+      <c r="O65" s="3">
         <v>0.36</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:15">
       <c r="A66" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B66" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C66" s="1">
         <v>20</v>
       </c>
       <c r="D66" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E66">
         <v>120</v>
@@ -3120,37 +3703,37 @@
       <c r="I66">
         <v>4</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="3">
         <v>0.96</v>
       </c>
       <c r="K66" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L66">
         <v>2202990</v>
       </c>
-      <c r="M66" s="3">
+      <c r="M66" s="4">
         <v>44882</v>
       </c>
       <c r="N66">
         <v>4</v>
       </c>
-      <c r="O66" s="2">
+      <c r="O66" s="3">
         <v>0.96</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:15">
       <c r="A67" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B67" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C67" s="1">
         <v>20</v>
       </c>
       <c r="D67" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E67">
         <v>600</v>
@@ -3161,37 +3744,37 @@
       <c r="I67">
         <v>1</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="3">
         <v>1.2</v>
       </c>
       <c r="K67" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L67">
         <v>2202990</v>
       </c>
-      <c r="M67" s="3">
+      <c r="M67" s="4">
         <v>44882</v>
       </c>
       <c r="N67">
         <v>1</v>
       </c>
-      <c r="O67" s="2">
+      <c r="O67" s="3">
         <v>1.2</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:15">
       <c r="A68" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B68" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C68" s="1">
         <v>70</v>
       </c>
       <c r="D68" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E68">
         <v>290</v>
@@ -3202,37 +3785,37 @@
       <c r="I68">
         <v>1</v>
       </c>
-      <c r="J68" s="2">
-        <v>0.40310000000000001</v>
+      <c r="J68" s="3">
+        <v>0.4031</v>
       </c>
       <c r="K68" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L68">
         <v>2202644</v>
       </c>
-      <c r="M68" s="3">
+      <c r="M68" s="4">
         <v>44848</v>
       </c>
       <c r="N68">
         <v>1</v>
       </c>
-      <c r="O68" s="2">
-        <v>0.40310000000000001</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O68" s="3">
+        <v>0.4031</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15">
       <c r="A69" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B69" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C69" s="1">
         <v>70</v>
       </c>
       <c r="D69" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E69">
         <v>290</v>
@@ -3243,37 +3826,37 @@
       <c r="I69">
         <v>1</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="3">
         <v>0.3886</v>
       </c>
       <c r="K69" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L69">
         <v>2202644</v>
       </c>
-      <c r="M69" s="3">
+      <c r="M69" s="4">
         <v>44848</v>
       </c>
       <c r="N69">
         <v>1</v>
       </c>
-      <c r="O69" s="2">
+      <c r="O69" s="3">
         <v>0.3886</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:15">
       <c r="A70" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B70" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C70" s="1">
         <v>70</v>
       </c>
       <c r="D70" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E70">
         <v>1160</v>
@@ -3284,26 +3867,27 @@
       <c r="I70">
         <v>1</v>
       </c>
-      <c r="J70" s="2">
-        <v>0.73080000000000001</v>
+      <c r="J70" s="3">
+        <v>0.7308</v>
       </c>
       <c r="K70" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L70">
         <v>2202644</v>
       </c>
-      <c r="M70" s="3">
+      <c r="M70" s="4">
         <v>44848</v>
       </c>
       <c r="N70">
         <v>1</v>
       </c>
-      <c r="O70" s="2">
-        <v>0.73080000000000001</v>
+      <c r="O70" s="3">
+        <v>0.7308</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>